<commit_message>
Translate retargeting headlines into Romanian
Adds Romanian translations for 5 follow-up/retargeting ad headlines
in YOUnity brand voice — empowering, spiritually resonant, direct.

https://claude.ai/code/session_01Bucp1gXMUaJVjdSyBMQ25o
</commit_message>
<xml_diff>
--- a/Blueprint/brg-cc-k3/brg-cc-k3 Facebook Ad Copy.xlsx
+++ b/Blueprint/brg-cc-k3/brg-cc-k3 Facebook Ad Copy.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -63,13 +63,21 @@
       <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BDD7EE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -91,7 +99,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -119,6 +127,12 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -381,7 +395,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I91"/>
+  <dimension ref="B2:I98"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.515625" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="5" min="1" max="1"/>
@@ -1790,6 +1804,83 @@
       </c>
     </row>
     <row r="92" ht="3.75" customHeight="1" s="6"/>
+    <row r="93" ht="20" customHeight="1" s="6">
+      <c r="B93" s="10" t="inlineStr">
+        <is>
+          <t>RETARGETING / FOLLOW-UP HEADLINES — Romanian Translations</t>
+        </is>
+      </c>
+      <c r="C93" s="10" t="inlineStr">
+        <is>
+          <t>Original (English)</t>
+        </is>
+      </c>
+      <c r="D93" s="10" t="inlineStr">
+        <is>
+          <t>Romanian</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="22" customHeight="1" s="6">
+      <c r="C94" s="11" t="inlineStr">
+        <is>
+          <t>Go Deeper Into The Human Blueprint</t>
+        </is>
+      </c>
+      <c r="D94" s="11" t="inlineStr">
+        <is>
+          <t>Pătrunzi Mai Adânc În Blueprintul Uman</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="22" customHeight="1" s="6">
+      <c r="C95" s="11" t="inlineStr">
+        <is>
+          <t>Make The Shift Real This Time</t>
+        </is>
+      </c>
+      <c r="D95" s="11" t="inlineStr">
+        <is>
+          <t>Fă Schimbarea Reală De Data Aceasta</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="22" customHeight="1" s="6">
+      <c r="C96" s="11" t="inlineStr">
+        <is>
+          <t>Come Back To Your Center</t>
+        </is>
+      </c>
+      <c r="D96" s="11" t="inlineStr">
+        <is>
+          <t>Revino La Centrul Tău</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="22" customHeight="1" s="6">
+      <c r="C97" s="11" t="inlineStr">
+        <is>
+          <t>Go Beyond The Free Training</t>
+        </is>
+      </c>
+      <c r="D97" s="11" t="inlineStr">
+        <is>
+          <t>Mergi Dincolo De Seria Gratuită</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="22" customHeight="1" s="6">
+      <c r="C98" s="11" t="inlineStr">
+        <is>
+          <t>Turn Insight Into Inner Change</t>
+        </is>
+      </c>
+      <c r="D98" s="11" t="inlineStr">
+        <is>
+          <t>Transformă Revelația În Schimbare Interioară</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>